<commit_message>
live update 14:16:19 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -461,13 +461,13 @@
     <col width="6" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="21" customWidth="1" min="23" max="23"/>
     <col width="23" customWidth="1" min="24" max="24"/>
-    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="30" customWidth="1" min="28" max="28"/>
@@ -736,6 +736,536 @@
         </is>
       </c>
       <c r="AD2" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>14:12:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.5446</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.5397999999999999</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="V3" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>0.07458773136138916</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>-11.89</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.6657999999999999</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.6004</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>11300</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="V4" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>0.1957922267913818</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>-13.87</v>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP1 MINLATE $86@0.440</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>14:14:03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.6135</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6150</v>
+      </c>
+      <c r="K5" t="n">
+        <v>8600</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="V5" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>29.39</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>14:15:47</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.6135</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6150</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8600</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="V6" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>14:15:58</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.5748</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.5548999999999999</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="K7" t="n">
+        <v>11350</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>12</v>
+      </c>
+      <c r="O7" t="n">
+        <v>7</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="V7" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
         <is>
           <t>Ursa</t>
         </is>
@@ -752,7 +1282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -888,6 +1418,57 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>195.7442204545454</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>0.6657922267913818</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.1957922267913818</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:21:24 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1271,6 +1271,422 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>14:17:11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.5748</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.5548999999999999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>3750</v>
+      </c>
+      <c r="K8" t="n">
+        <v>11350</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>12</v>
+      </c>
+      <c r="O8" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="V8" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14:17:22</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.7427</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.6388</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>9250</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>17</v>
+      </c>
+      <c r="O9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P9" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="V9" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14:19:06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.7775</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.6562</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5250</v>
+      </c>
+      <c r="K10" t="n">
+        <v>9350</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>22</v>
+      </c>
+      <c r="O10" t="n">
+        <v>12</v>
+      </c>
+      <c r="P10" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="V10" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14:20:31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0.6324</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.5837</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2550</v>
+      </c>
+      <c r="K11" t="n">
+        <v>12100</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>23</v>
+      </c>
+      <c r="O11" t="n">
+        <v>17</v>
+      </c>
+      <c r="P11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>2</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="V11" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:26:30 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AD16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1687,6 +1687,526 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>14:22:37</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.6324</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.5837</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2550</v>
+      </c>
+      <c r="K12" t="n">
+        <v>12100</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>23</v>
+      </c>
+      <c r="O12" t="n">
+        <v>17</v>
+      </c>
+      <c r="P12" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="V12" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>-2.01</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>14:22:48</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.5905</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.5627</v>
+      </c>
+      <c r="J13" t="n">
+        <v>6350</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3800</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>24</v>
+      </c>
+      <c r="O13" t="n">
+        <v>21</v>
+      </c>
+      <c r="P13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R13" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="V13" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>-3.96</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>14:23:51</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.7364000000000001</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.6357</v>
+      </c>
+      <c r="J14" t="n">
+        <v>450</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1700</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>26</v>
+      </c>
+      <c r="O14" t="n">
+        <v>24</v>
+      </c>
+      <c r="P14" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>3</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="V14" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>14:25:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>5-5</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.7364000000000001</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0.6357</v>
+      </c>
+      <c r="J15" t="n">
+        <v>450</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1700</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>26</v>
+      </c>
+      <c r="O15" t="n">
+        <v>24</v>
+      </c>
+      <c r="P15" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="V15" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>-13.82</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>14:25:16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>5-5</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.6067</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0.5709</v>
+      </c>
+      <c r="J16" t="n">
+        <v>550</v>
+      </c>
+      <c r="K16" t="n">
+        <v>4250</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>28</v>
+      </c>
+      <c r="O16" t="n">
+        <v>29</v>
+      </c>
+      <c r="P16" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>4</v>
+      </c>
+      <c r="R16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V16" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>-11.84</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:31:36 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -66,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +75,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD16"/>
+  <dimension ref="A1:AD21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2208,537 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>14:27:02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.6067</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0.5709</v>
+      </c>
+      <c r="J17" t="n">
+        <v>550</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4250</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>28</v>
+      </c>
+      <c r="O17" t="n">
+        <v>29</v>
+      </c>
+      <c r="P17" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>4</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="V17" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>14:27:13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>11</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.5164</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0.5256999999999999</v>
+      </c>
+      <c r="J18" t="n">
+        <v>6850</v>
+      </c>
+      <c r="K18" t="n">
+        <v>8250</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>29</v>
+      </c>
+      <c r="O18" t="n">
+        <v>34</v>
+      </c>
+      <c r="P18" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="V18" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:MINLATE@0.440x196</t>
+        </is>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14:28:57</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>6-6</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.5164</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0.5256999999999999</v>
+      </c>
+      <c r="J19" t="n">
+        <v>6850</v>
+      </c>
+      <c r="K19" t="n">
+        <v>8250</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>29</v>
+      </c>
+      <c r="O19" t="n">
+        <v>34</v>
+      </c>
+      <c r="P19" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>4</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="V19" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>58.94</v>
+      </c>
+      <c r="AB19" s="4" t="inlineStr">
+        <is>
+          <t>SELL MAP1 MINLATE P/L:$+35.23</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:29:08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>6-6</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.4854</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>0.5102</v>
+      </c>
+      <c r="J20" t="n">
+        <v>4750</v>
+      </c>
+      <c r="K20" t="n">
+        <v>11850</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>32</v>
+      </c>
+      <c r="O20" t="n">
+        <v>39</v>
+      </c>
+      <c r="P20" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>4</v>
+      </c>
+      <c r="R20" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="V20" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X20" s="3" t="n">
+        <v>0.1346157443523407</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>17.84</v>
+      </c>
+      <c r="AB20" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP1 Ursa $51@0.350</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:30:42</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>13</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>7-6</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0.6421</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0.5886</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>37</v>
+      </c>
+      <c r="O21" t="n">
+        <v>43</v>
+      </c>
+      <c r="P21" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>5</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="V21" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2218,7 +2750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2232,8 +2764,8 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2402,6 +2934,108 @@
         <v>0.1957922267913818</v>
       </c>
       <c r="M3" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>14:28:57</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>195.7442204545454</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>0.5163925886154175</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>-0.1336074113845825</v>
+      </c>
+      <c r="M4" s="8" t="n">
+        <v>35.23395968181818</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>14:29:08</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>144.6360388571429</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>0.5146157443523407</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.585</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0.1346157443523407</v>
+      </c>
+      <c r="M5" s="7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
live update 14:36:42 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD21"/>
+  <dimension ref="A1:AD26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2739,6 +2739,526 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>14:32:49</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>14</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.7334000000000001</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0.6342</v>
+      </c>
+      <c r="J22" t="n">
+        <v>6750</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1600</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>42</v>
+      </c>
+      <c r="O22" t="n">
+        <v>45</v>
+      </c>
+      <c r="P22" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>5</v>
+      </c>
+      <c r="R22" t="n">
+        <v>2</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="V22" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-2.79</v>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>14:34:34</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>14</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>9-6</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.7334000000000001</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0.6342</v>
+      </c>
+      <c r="J23" t="n">
+        <v>6750</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1600</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>42</v>
+      </c>
+      <c r="O23" t="n">
+        <v>45</v>
+      </c>
+      <c r="P23" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>5</v>
+      </c>
+      <c r="R23" t="n">
+        <v>2</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="V23" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>-12.75</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>14:34:45</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>9-6</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0.8032</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0.6691</v>
+      </c>
+      <c r="J24" t="n">
+        <v>9500</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1700</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>47</v>
+      </c>
+      <c r="O24" t="n">
+        <v>47</v>
+      </c>
+      <c r="P24" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>6</v>
+      </c>
+      <c r="R24" t="n">
+        <v>3</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V24" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z24" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>-10.77</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>14:35:48</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>16</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>10-6</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0.8613</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0.6982</v>
+      </c>
+      <c r="J25" t="n">
+        <v>12250</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4300</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>52</v>
+      </c>
+      <c r="O25" t="n">
+        <v>49</v>
+      </c>
+      <c r="P25" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>4</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V25" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z25" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>-16.56</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>14:35:59</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>16</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>10-6</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0.8613</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0.6982</v>
+      </c>
+      <c r="J26" t="n">
+        <v>12250</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4300</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>52</v>
+      </c>
+      <c r="O26" t="n">
+        <v>49</v>
+      </c>
+      <c r="P26" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>6</v>
+      </c>
+      <c r="R26" t="n">
+        <v>4</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V26" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z26" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>-11.68</v>
+      </c>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:41:46 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -66,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -76,6 +82,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD26"/>
+  <dimension ref="A1:AD30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3259,6 +3266,429 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>14:37:03</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>16</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>11-6</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0.8613</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0.6982</v>
+      </c>
+      <c r="J27" t="n">
+        <v>12250</v>
+      </c>
+      <c r="K27" t="n">
+        <v>4300</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>52</v>
+      </c>
+      <c r="O27" t="n">
+        <v>49</v>
+      </c>
+      <c r="P27" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>6</v>
+      </c>
+      <c r="R27" t="n">
+        <v>4</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V27" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z27" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>-6.43</v>
+      </c>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:37:14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>17</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>11-6</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0.9238</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0.7294</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3600</v>
+      </c>
+      <c r="K28" t="n">
+        <v>8800</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>57</v>
+      </c>
+      <c r="O28" t="n">
+        <v>49</v>
+      </c>
+      <c r="P28" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>6</v>
+      </c>
+      <c r="R28" t="n">
+        <v>5</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="V28" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198; MAP1:Ursa@0.350x145</t>
+        </is>
+      </c>
+      <c r="Z28" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>-8.41</v>
+      </c>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14:39:08</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>11-7</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>0.9716</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0.7533</v>
+      </c>
+      <c r="J29" t="n">
+        <v>6150</v>
+      </c>
+      <c r="K29" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>62</v>
+      </c>
+      <c r="O29" t="n">
+        <v>52</v>
+      </c>
+      <c r="P29" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>7</v>
+      </c>
+      <c r="R29" t="n">
+        <v>6</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="U29" s="2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="V29" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z29" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AB29" s="4" t="inlineStr">
+        <is>
+          <t>SELL MAP1 Ursa P/L:$-27.48</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:41:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>19</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>11-8</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1650</v>
+      </c>
+      <c r="K30" t="n">
+        <v>7950</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>66</v>
+      </c>
+      <c r="O30" t="n">
+        <v>57</v>
+      </c>
+      <c r="P30" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>7</v>
+      </c>
+      <c r="R30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U30" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V30" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X30" s="2" t="n">
+        <v>-0.007040214538574258</v>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z30" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>31.71</v>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3270,7 +3700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3282,10 +3712,10 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3557,6 +3987,57 @@
       </c>
       <c r="M5" s="7" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>14:39:08</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>144.6360388571429</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.02837634086608887</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.585</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>-0.1616236591339111</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>-27.48084738285714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
live update 14:46:51 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
+++ b/data/live_logs/live_cs2-minlat-ursa-2026-04-03_20260403_131052.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD30"/>
+  <dimension ref="A1:AD33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3689,6 +3689,327 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:44:02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>20</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>12-8</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0.9085</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0.7217</v>
+      </c>
+      <c r="J31" t="n">
+        <v>11450</v>
+      </c>
+      <c r="K31" t="n">
+        <v>2050</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>67</v>
+      </c>
+      <c r="O31" t="n">
+        <v>59</v>
+      </c>
+      <c r="P31" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>7</v>
+      </c>
+      <c r="R31" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="T31" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="V31" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X31" s="2" t="n">
+        <v>0.008458709716796881</v>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z31" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>25.76</v>
+      </c>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:45:36</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>20</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>12-9</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0.9085</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0.7217</v>
+      </c>
+      <c r="J32" t="n">
+        <v>11450</v>
+      </c>
+      <c r="K32" t="n">
+        <v>2050</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>67</v>
+      </c>
+      <c r="O32" t="n">
+        <v>59</v>
+      </c>
+      <c r="P32" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>7</v>
+      </c>
+      <c r="R32" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T32" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V32" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X32" s="2" t="n">
+        <v>-0.03845870971679688</v>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z32" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>29.73</v>
+      </c>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:45:48</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>21</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>12-9</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0.9722</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0.7536</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3050</v>
+      </c>
+      <c r="K33" t="n">
+        <v>8750</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>72</v>
+      </c>
+      <c r="O33" t="n">
+        <v>62</v>
+      </c>
+      <c r="P33" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>8</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V33" t="n">
+        <v>6422.0707</v>
+      </c>
+      <c r="X33" s="2" t="n">
+        <v>0.04215276956558225</v>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>WINNER:MINLATE@0.340x198</t>
+        </is>
+      </c>
+      <c r="Z33" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>29.73</v>
+      </c>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>MINLATE</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>